<commit_message>
removed Thread.sleep from VaultPointsWithDiscountTest
</commit_message>
<xml_diff>
--- a/src/com/baublebar/data/TestCases.xlsx
+++ b/src/com/baublebar/data/TestCases.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="460" windowWidth="27100" windowHeight="15820" activeTab="1"/>
+    <workbookView xWindow="1700" yWindow="460" windowWidth="27100" windowHeight="15820" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="92">
   <si>
     <t>TCID</t>
   </si>
@@ -166,9 +166,6 @@
     <t>ProductName</t>
   </si>
   <si>
-    <t>ice-dog-tag-layered-pendant-necklace</t>
-  </si>
-  <si>
     <t>What's New</t>
   </si>
   <si>
@@ -265,10 +262,28 @@
     <t>EarnVaultPointTest</t>
   </si>
   <si>
-    <t>pave-sputnik-ear-jackets-earring</t>
-  </si>
-  <si>
-    <t>VaultPointWithDicountTest</t>
+    <t>CCExpirMonth</t>
+  </si>
+  <si>
+    <t>CCExpirYear</t>
+  </si>
+  <si>
+    <t>starry-avatar-cuff-bracelet</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>2017</t>
+  </si>
+  <si>
+    <t>bahama-tassel-drops-earrings</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>BBENG</t>
   </si>
   <si>
     <t>VaultPointAmount</t>
@@ -277,7 +292,16 @@
     <t>DiscountCode</t>
   </si>
   <si>
-    <t>BBENG</t>
+    <t>PaginationTest</t>
+  </si>
+  <si>
+    <t>What'sNew</t>
+  </si>
+  <si>
+    <t>VaultPointsWithDicountTest</t>
+  </si>
+  <si>
+    <t>starburst-studs-earrings</t>
   </si>
 </sst>
 </file>
@@ -744,7 +768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -869,7 +893,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
         <v>3</v>
@@ -877,7 +901,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C16" t="s">
         <v>3</v>
@@ -885,7 +909,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C17" t="s">
         <v>3</v>
@@ -893,7 +917,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C18" t="s">
         <v>3</v>
@@ -901,7 +925,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C19" t="s">
         <v>3</v>
@@ -909,7 +933,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C20" t="s">
         <v>3</v>
@@ -917,9 +941,17 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>88</v>
+      </c>
+      <c r="C22" t="s">
         <v>3</v>
       </c>
     </row>
@@ -931,7 +963,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M98"/>
+  <dimension ref="A1:O109"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.33203125" customWidth="1"/>
@@ -947,6 +979,8 @@
     <col min="11" max="11" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="20.1640625" customWidth="1"/>
     <col min="13" max="13" width="10.83203125" customWidth="1"/>
+    <col min="14" max="14" width="13.5" customWidth="1"/>
+    <col min="15" max="15" width="9.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -1204,7 +1238,7 @@
         <v>3</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C47" s="12"/>
     </row>
@@ -1217,7 +1251,7 @@
       </c>
       <c r="C48" s="12"/>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49" s="12" t="s">
         <v>3</v>
       </c>
@@ -1226,7 +1260,7 @@
       </c>
       <c r="C49" s="12"/>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A50" s="12" t="s">
         <v>3</v>
       </c>
@@ -1235,7 +1269,7 @@
       </c>
       <c r="C50" s="12"/>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A51" s="12" t="s">
         <v>3</v>
       </c>
@@ -1244,7 +1278,7 @@
       </c>
       <c r="C51" s="12"/>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52" s="12" t="s">
         <v>3</v>
       </c>
@@ -1252,7 +1286,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53" s="12" t="s">
         <v>3</v>
       </c>
@@ -1260,7 +1294,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54" s="12" t="s">
         <v>3</v>
       </c>
@@ -1268,12 +1302,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A56" s="14" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A57" s="12" t="s">
         <v>2</v>
       </c>
@@ -1284,16 +1318,16 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" s="12" t="s">
         <v>3</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C58" s="12"/>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59" s="12" t="s">
         <v>3</v>
       </c>
@@ -1302,7 +1336,7 @@
       </c>
       <c r="C59" s="12"/>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A60" s="12" t="s">
         <v>3</v>
       </c>
@@ -1311,7 +1345,7 @@
       </c>
       <c r="C60" s="12"/>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61" s="12" t="s">
         <v>3</v>
       </c>
@@ -1319,8 +1353,9 @@
         <v>34</v>
       </c>
       <c r="C61" s="12"/>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="O61" s="3"/>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A62" s="12" t="s">
         <v>3</v>
       </c>
@@ -1329,7 +1364,7 @@
       </c>
       <c r="C62" s="12"/>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A63" s="12" t="s">
         <v>3</v>
       </c>
@@ -1337,7 +1372,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A64" s="12" t="s">
         <v>3</v>
       </c>
@@ -1345,7 +1380,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A65" s="12" t="s">
         <v>3</v>
       </c>
@@ -1353,7 +1388,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A66" s="12" t="s">
         <v>15</v>
       </c>
@@ -1361,12 +1396,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A68" s="14" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A69" s="12" t="s">
         <v>2</v>
       </c>
@@ -1374,86 +1409,98 @@
         <v>45</v>
       </c>
       <c r="C69" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D69" t="s">
         <v>5</v>
       </c>
       <c r="E69" t="s">
+        <v>49</v>
+      </c>
+      <c r="F69" t="s">
+        <v>60</v>
+      </c>
+      <c r="G69" t="s">
+        <v>59</v>
+      </c>
+      <c r="H69" t="s">
         <v>50</v>
       </c>
-      <c r="F69" t="s">
-        <v>61</v>
-      </c>
-      <c r="G69" t="s">
-        <v>60</v>
-      </c>
-      <c r="H69" t="s">
+      <c r="I69" t="s">
         <v>51</v>
       </c>
-      <c r="I69" t="s">
+      <c r="J69" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="J69" s="15" t="s">
+      <c r="K69" t="s">
         <v>53</v>
       </c>
-      <c r="K69" t="s">
+      <c r="L69" t="s">
+        <v>64</v>
+      </c>
+      <c r="M69" t="s">
+        <v>65</v>
+      </c>
+      <c r="N69" t="s">
+        <v>78</v>
+      </c>
+      <c r="O69" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" ht="18" x14ac:dyDescent="0.2">
+      <c r="A70" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C70" t="s">
         <v>54</v>
-      </c>
-      <c r="L69" t="s">
-        <v>65</v>
-      </c>
-      <c r="M69" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="70" spans="1:13" ht="18" x14ac:dyDescent="0.2">
-      <c r="A70" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C70" t="s">
-        <v>55</v>
       </c>
       <c r="D70" t="s">
         <v>18</v>
       </c>
       <c r="E70" t="s">
+        <v>55</v>
+      </c>
+      <c r="F70" t="s">
         <v>56</v>
       </c>
-      <c r="F70" t="s">
+      <c r="G70" t="s">
         <v>57</v>
       </c>
-      <c r="G70" t="s">
+      <c r="H70" t="s">
         <v>58</v>
       </c>
-      <c r="H70" t="s">
-        <v>59</v>
-      </c>
       <c r="I70" t="s">
+        <v>61</v>
+      </c>
+      <c r="J70" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="K70" t="s">
         <v>62</v>
       </c>
-      <c r="J70" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="K70" t="s">
-        <v>63</v>
-      </c>
       <c r="L70" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="M70" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="M70" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N70" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="O70" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A72" s="11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A73" s="12" t="s">
         <v>2</v>
       </c>
@@ -1461,32 +1508,32 @@
         <v>45</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A74" s="12" t="s">
         <v>3</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A76" s="11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A80" s="11" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A80" s="11" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
@@ -1494,7 +1541,7 @@
         <v>2</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
@@ -1502,12 +1549,12 @@
         <v>3</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
@@ -1523,12 +1570,12 @@
         <v>3</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
@@ -1544,12 +1591,12 @@
         <v>3</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
@@ -1565,16 +1612,16 @@
         <v>3</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
-        <v>80</v>
+      <c r="A96" s="11" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A97" s="12" t="s">
+      <c r="A97" t="s">
         <v>2</v>
       </c>
       <c r="B97" s="3" t="s">
@@ -1587,18 +1634,18 @@
         <v>5</v>
       </c>
       <c r="E97" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F97" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A98" s="12" t="s">
+      <c r="A98" t="s">
         <v>3</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C98" s="5" t="s">
         <v>17</v>
@@ -1606,11 +1653,88 @@
       <c r="D98" t="s">
         <v>18</v>
       </c>
-      <c r="E98">
-        <v>1</v>
+      <c r="E98" s="3" t="s">
+        <v>84</v>
       </c>
       <c r="F98" t="s">
-        <v>83</v>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A100" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>2</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>3</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>3</v>
+      </c>
+      <c r="B103" s="13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>3</v>
+      </c>
+      <c r="B104" s="13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>3</v>
+      </c>
+      <c r="B105" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>3</v>
+      </c>
+      <c r="B106" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>3</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>3</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>3</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added AddItemsTest And Update VaultPointsWithDiscountTest
</commit_message>
<xml_diff>
--- a/src/com/baublebar/data/TestCases.xlsx
+++ b/src/com/baublebar/data/TestCases.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="101">
   <si>
     <t>TCID</t>
   </si>
@@ -280,46 +280,55 @@
     <t>1</t>
   </si>
   <si>
+    <t>VaultPointAmount</t>
+  </si>
+  <si>
+    <t>DiscountCode</t>
+  </si>
+  <si>
+    <t>PaginationTest</t>
+  </si>
+  <si>
+    <t>VaultPointsWithDicountTest</t>
+  </si>
+  <si>
+    <t>starburst-studs-earrings</t>
+  </si>
+  <si>
+    <t>necklaces</t>
+  </si>
+  <si>
+    <t>earrings</t>
+  </si>
+  <si>
+    <t>bracelets</t>
+  </si>
+  <si>
+    <t>rings</t>
+  </si>
+  <si>
+    <t>personalized</t>
+  </si>
+  <si>
+    <t>whats-new/just-added</t>
+  </si>
+  <si>
+    <t>pave-droplet-ear-crawlers-earrings</t>
+  </si>
+  <si>
+    <t>ProductName1</t>
+  </si>
+  <si>
+    <t>ProductName2</t>
+  </si>
+  <si>
+    <t>AddItemsTest</t>
+  </si>
+  <si>
+    <t>RemoveItemFromShoppingCartTest</t>
+  </si>
+  <si>
     <t>BBENG</t>
-  </si>
-  <si>
-    <t>VaultPointAmount</t>
-  </si>
-  <si>
-    <t>DiscountCode</t>
-  </si>
-  <si>
-    <t>PaginationTest</t>
-  </si>
-  <si>
-    <t>VaultPointsWithDicountTest</t>
-  </si>
-  <si>
-    <t>starburst-studs-earrings</t>
-  </si>
-  <si>
-    <t>necklaces</t>
-  </si>
-  <si>
-    <t>earrings</t>
-  </si>
-  <si>
-    <t>bracelets</t>
-  </si>
-  <si>
-    <t>rings</t>
-  </si>
-  <si>
-    <t>personalized</t>
-  </si>
-  <si>
-    <t>whats-new/just-added</t>
-  </si>
-  <si>
-    <t>RemoveItemTest</t>
-  </si>
-  <si>
-    <t>pave-droplet-ear-crawlers-earrings</t>
   </si>
 </sst>
 </file>
@@ -786,7 +795,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -959,7 +968,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C21" t="s">
         <v>3</v>
@@ -967,7 +976,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C22" t="s">
         <v>3</v>
@@ -975,9 +984,17 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>98</v>
+      </c>
+      <c r="C24" t="s">
         <v>3</v>
       </c>
     </row>
@@ -989,12 +1006,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O111"/>
+  <dimension ref="A1:O115"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.33203125" customWidth="1"/>
+    <col min="1" max="1" width="27.33203125" customWidth="1"/>
     <col min="2" max="2" width="34.6640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="23.33203125" customWidth="1"/>
+    <col min="3" max="3" width="26.6640625" customWidth="1"/>
     <col min="4" max="4" width="15.33203125" customWidth="1"/>
     <col min="5" max="5" width="19.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
@@ -1229,7 +1246,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>29</v>
@@ -1638,12 +1655,12 @@
         <v>3</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.2">
@@ -1660,10 +1677,10 @@
         <v>5</v>
       </c>
       <c r="E97" t="s">
+        <v>84</v>
+      </c>
+      <c r="F97" t="s">
         <v>85</v>
-      </c>
-      <c r="F97" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.2">
@@ -1671,7 +1688,7 @@
         <v>3</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C98" s="5" t="s">
         <v>17</v>
@@ -1683,12 +1700,12 @@
         <v>83</v>
       </c>
       <c r="F98" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.2">
@@ -1704,7 +1721,7 @@
         <v>3</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.2">
@@ -1712,7 +1729,7 @@
         <v>3</v>
       </c>
       <c r="B103" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.2">
@@ -1720,7 +1737,7 @@
         <v>3</v>
       </c>
       <c r="B104" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.2">
@@ -1728,7 +1745,7 @@
         <v>3</v>
       </c>
       <c r="B105" s="13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.2">
@@ -1736,7 +1753,7 @@
         <v>3</v>
       </c>
       <c r="B106" s="13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.2">
@@ -1744,7 +1761,7 @@
         <v>3</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.2">
@@ -1753,8 +1770,8 @@
       <c r="J108"/>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
-        <v>96</v>
+      <c r="A109" s="11" t="s">
+        <v>99</v>
       </c>
       <c r="B109"/>
       <c r="I109" s="15"/>
@@ -1775,7 +1792,34 @@
         <v>3</v>
       </c>
       <c r="B111" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A113" s="11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>2</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C114" t="s">
         <v>97</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>3</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C115" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Remove from shopping cart
Update Remove from shopping cart
</commit_message>
<xml_diff>
--- a/src/com/baublebar/data/TestCases.xlsx
+++ b/src/com/baublebar/data/TestCases.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="460" windowWidth="20260" windowHeight="15820"/>
+    <workbookView xWindow="1700" yWindow="460" windowWidth="27100" windowHeight="15820" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="104">
   <si>
     <t>TCID</t>
   </si>
@@ -274,61 +274,70 @@
     <t>starry-avatar-cuff-bracelet</t>
   </si>
   <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>2017</t>
+  </si>
+  <si>
     <t>VaultPointsWithDiscountTest</t>
   </si>
   <si>
+    <t>bahama-tassel-drops-earrings</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>BBENG</t>
+  </si>
+  <si>
     <t>VaultPointAmount</t>
   </si>
   <si>
     <t>DiscountCode</t>
   </si>
   <si>
-    <t>roma-studs-earrings</t>
-  </si>
-  <si>
-    <t>BBENG</t>
-  </si>
-  <si>
-    <t>AddItemsTest</t>
-  </si>
-  <si>
     <t>PaginationTest</t>
   </si>
   <si>
+    <t>personalized</t>
+  </si>
+  <si>
+    <t>rings</t>
+  </si>
+  <si>
+    <t>earrings</t>
+  </si>
+  <si>
+    <t>bracelets</t>
+  </si>
+  <si>
+    <t>necklaces</t>
+  </si>
+  <si>
+    <t>whats-new/just-added</t>
+  </si>
+  <si>
     <t>RemoveItemFromShoppingCartTest</t>
   </si>
   <si>
     <t>ProductName1</t>
   </si>
   <si>
+    <t>ProductName3</t>
+  </si>
+  <si>
     <t>ProductName2</t>
   </si>
   <si>
-    <t>brunello-studs-earrings</t>
-  </si>
-  <si>
-    <t>whats-new/just-added</t>
-  </si>
-  <si>
-    <t>necklaces</t>
-  </si>
-  <si>
-    <t>earrings</t>
-  </si>
-  <si>
-    <t>bracelets</t>
-  </si>
-  <si>
-    <t>rings</t>
-  </si>
-  <si>
-    <t>personalized/view-all</t>
-  </si>
-  <si>
-    <t>demi-tassel-bib-necklace</t>
-  </si>
-  <si>
-    <t>8</t>
+    <t>tundra-drops-earrings</t>
+  </si>
+  <si>
+    <t>tundra-studs-earrings</t>
+  </si>
+  <si>
+    <t>starburst-studs-earrings</t>
   </si>
 </sst>
 </file>
@@ -795,10 +804,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="1" max="1" width="28.33203125" customWidth="1"/>
     <col min="2" max="2" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -968,7 +977,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C21" t="s">
         <v>3</v>
@@ -976,7 +985,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C22" t="s">
         <v>3</v>
@@ -984,17 +993,9 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="C23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>89</v>
-      </c>
-      <c r="C24" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1006,13 +1007,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O115"/>
+  <dimension ref="A1:O113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="34.6640625" style="3" customWidth="1"/>
     <col min="3" max="3" width="23.33203125" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
     <col min="5" max="5" width="19.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="15.1640625" customWidth="1"/>
@@ -1023,6 +1024,7 @@
     <col min="12" max="12" width="20.1640625" customWidth="1"/>
     <col min="13" max="13" width="10.83203125" customWidth="1"/>
     <col min="14" max="14" width="13.5" customWidth="1"/>
+    <col min="15" max="15" width="9.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -1293,7 +1295,7 @@
       </c>
       <c r="C48" s="12"/>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49" s="12" t="s">
         <v>3</v>
       </c>
@@ -1302,7 +1304,7 @@
       </c>
       <c r="C49" s="12"/>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A50" s="12" t="s">
         <v>3</v>
       </c>
@@ -1311,7 +1313,7 @@
       </c>
       <c r="C50" s="12"/>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A51" s="12" t="s">
         <v>3</v>
       </c>
@@ -1320,7 +1322,7 @@
       </c>
       <c r="C51" s="12"/>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52" s="12" t="s">
         <v>3</v>
       </c>
@@ -1328,7 +1330,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53" s="12" t="s">
         <v>3</v>
       </c>
@@ -1336,7 +1338,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54" s="12" t="s">
         <v>3</v>
       </c>
@@ -1344,12 +1346,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A56" s="14" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A57" s="12" t="s">
         <v>2</v>
       </c>
@@ -1360,7 +1362,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" s="12" t="s">
         <v>3</v>
       </c>
@@ -1369,7 +1371,7 @@
       </c>
       <c r="C58" s="12"/>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59" s="12" t="s">
         <v>3</v>
       </c>
@@ -1378,7 +1380,7 @@
       </c>
       <c r="C59" s="12"/>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A60" s="12" t="s">
         <v>3</v>
       </c>
@@ -1387,7 +1389,7 @@
       </c>
       <c r="C60" s="12"/>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61" s="12" t="s">
         <v>3</v>
       </c>
@@ -1395,8 +1397,9 @@
         <v>34</v>
       </c>
       <c r="C61" s="12"/>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="O61" s="3"/>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A62" s="12" t="s">
         <v>3</v>
       </c>
@@ -1405,7 +1408,7 @@
       </c>
       <c r="C62" s="12"/>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A63" s="12" t="s">
         <v>3</v>
       </c>
@@ -1413,7 +1416,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A64" s="12" t="s">
         <v>3</v>
       </c>
@@ -1529,11 +1532,11 @@
       <c r="M70" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="N70">
-        <v>12</v>
-      </c>
-      <c r="O70">
-        <v>2019</v>
+      <c r="N70" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="O70" s="3" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.2">
@@ -1658,7 +1661,7 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" s="11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.2">
@@ -1666,19 +1669,19 @@
         <v>2</v>
       </c>
       <c r="B97" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C97" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C97" t="s">
+      <c r="D97" t="s">
         <v>5</v>
       </c>
-      <c r="D97" t="s">
-        <v>45</v>
-      </c>
       <c r="E97" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="F97" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.2">
@@ -1686,27 +1689,24 @@
         <v>3</v>
       </c>
       <c r="B98" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C98" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C98" t="s">
+      <c r="D98" t="s">
         <v>18</v>
       </c>
-      <c r="D98" t="s">
-        <v>99</v>
-      </c>
       <c r="E98" s="3" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="F98" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E99" s="3"/>
+        <v>87</v>
+      </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="11" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.2">
@@ -1714,10 +1714,7 @@
         <v>2</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="C101" t="s">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.2">
@@ -1725,39 +1722,47 @@
         <v>3</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C102" t="s">
-        <v>92</v>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>3</v>
+      </c>
+      <c r="B103" s="13" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A104" s="11" t="s">
-        <v>88</v>
+      <c r="A104" t="s">
+        <v>3</v>
+      </c>
+      <c r="B104" s="13" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>2</v>
-      </c>
-      <c r="B105" s="3" t="s">
-        <v>40</v>
+        <v>3</v>
+      </c>
+      <c r="B105" s="13" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>3</v>
       </c>
-      <c r="B106" s="3" t="s">
-        <v>93</v>
+      <c r="B106" s="13" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>94</v>
+        <v>37</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.2">
@@ -1765,52 +1770,48 @@
         <v>3</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A110" t="s">
-        <v>3</v>
-      </c>
-      <c r="B110" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A111" s="11" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
-        <v>3</v>
-      </c>
-      <c r="B111" s="3" t="s">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>2</v>
+      </c>
+      <c r="B112" s="3" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A113" s="11" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
-        <v>2</v>
-      </c>
-      <c r="B114" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
-        <v>3</v>
-      </c>
-      <c r="B115" s="3" t="s">
-        <v>85</v>
+      <c r="C112" t="s">
+        <v>100</v>
+      </c>
+      <c r="D112" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>3</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C113" t="s">
+        <v>102</v>
+      </c>
+      <c r="D113" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1819,6 +1820,7 @@
     <hyperlink ref="B31" r:id="rId2"/>
     <hyperlink ref="B7" r:id="rId3"/>
     <hyperlink ref="B15" r:id="rId4"/>
+    <hyperlink ref="C98" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293"/>

</xml_diff>

<commit_message>
Added Continue shopping test
Added Continue shopping test
</commit_message>
<xml_diff>
--- a/src/com/baublebar/data/TestCases.xlsx
+++ b/src/com/baublebar/data/TestCases.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="460" windowWidth="20260" windowHeight="15820" activeTab="1"/>
+    <workbookView xWindow="1100" yWindow="460" windowWidth="20260" windowHeight="15820"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="105">
   <si>
     <t>TCID</t>
   </si>
@@ -338,6 +338,9 @@
   </si>
   <si>
     <t>tundra-drops-earrings</t>
+  </si>
+  <si>
+    <t>ContinueShoppingTest</t>
   </si>
 </sst>
 </file>
@@ -804,7 +807,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -1007,6 +1010,14 @@
         <v>3</v>
       </c>
     </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
@@ -1015,7 +1026,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O115"/>
+  <dimension ref="A1:O119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
@@ -1834,6 +1845,27 @@
         <v>103</v>
       </c>
     </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A117" s="11" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
+        <v>2</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>3</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B11" r:id="rId1" display="cmaitri@yahoo.com"/>

</xml_diff>